<commit_message>
Update scorecard table styling
</commit_message>
<xml_diff>
--- a/Performance_Measures_R.xlsx
+++ b/Performance_Measures_R.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://palmbeachtpa-my.sharepoint.com/personal/skan_palmbeachmpo_org/Documents/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://palmbeachtpa-my.sharepoint.com/personal/skan_palmbeachmpo_org/Documents/Documents/Performance_Measures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="292" documentId="8_{6E25A293-DAE1-403C-87C6-760DEF9E0950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6B601152-700E-4F59-B056-B0454718EF4D}"/>
+  <xr:revisionPtr revIDLastSave="296" documentId="8_{6E25A293-DAE1-403C-87C6-760DEF9E0950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A95B10D5-944E-47D5-A2E3-BEF5848BC5F3}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{47865025-DE32-4D87-A21F-3C532F9D4B3D}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="10" xr2:uid="{47865025-DE32-4D87-A21F-3C532F9D4B3D}"/>
   </bookViews>
   <sheets>
     <sheet name="FATALITIES" sheetId="7" r:id="rId1"/>
@@ -23,7 +23,8 @@
     <sheet name="TTTR Index" sheetId="17" r:id="rId8"/>
     <sheet name="Int Reliability" sheetId="18" r:id="rId9"/>
     <sheet name="Non-Int Reliability" sheetId="19" r:id="rId10"/>
-    <sheet name="FATALITIES COMP" sheetId="3" state="hidden" r:id="rId11"/>
+    <sheet name="Scorecard_Safety" sheetId="21" r:id="rId11"/>
+    <sheet name="FATALITIES COMP" sheetId="3" state="hidden" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="91">
   <si>
     <t>Alachua</t>
   </si>
@@ -295,6 +296,30 @@
   </si>
   <si>
     <t>Target Good</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Non-motorized Fatalities and Serious Injuries</t>
+  </si>
+  <si>
+    <t>Serious Injury Rate</t>
+  </si>
+  <si>
+    <t>Serious Injuries</t>
+  </si>
+  <si>
+    <t>Fatal Crash Rate</t>
+  </si>
+  <si>
+    <t>Five_Year_Avg</t>
+  </si>
+  <si>
+    <t>Goal_Met</t>
+  </si>
+  <si>
+    <t>Metric</t>
   </si>
 </sst>
 </file>
@@ -1013,6 +1038,104 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B420F60-609B-4AA9-97E6-C695A4A591CA}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="43" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2">
+        <v>207.4</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C3">
+        <v>1.45</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4">
+        <v>812.2</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C5">
+        <v>5.73</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6">
+        <v>203.8</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DE6782D-92DC-4DC3-BB49-53C081EF8C06}">
   <dimension ref="A1:BP8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Added transit asset management charts and dashboard graphics
</commit_message>
<xml_diff>
--- a/Performance_Measures_R.xlsx
+++ b/Performance_Measures_R.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://palmbeachtpa-my.sharepoint.com/personal/skan_palmbeachmpo_org/Documents/Documents/Performance_Measures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="341" documentId="8_{6E25A293-DAE1-403C-87C6-760DEF9E0950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9AABFABA-DAC6-4814-8E88-1D26AEF7065E}"/>
+  <xr:revisionPtr revIDLastSave="400" documentId="8_{6E25A293-DAE1-403C-87C6-760DEF9E0950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E778E3EC-2CAB-4D41-8F8F-DF2C02C5FE69}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="10" activeTab="14" xr2:uid="{47865025-DE32-4D87-A21F-3C532F9D4B3D}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="13" xr2:uid="{47865025-DE32-4D87-A21F-3C532F9D4B3D}"/>
   </bookViews>
   <sheets>
     <sheet name="FATALITIES" sheetId="7" r:id="rId1"/>
@@ -23,12 +23,16 @@
     <sheet name="TTTR Index" sheetId="17" r:id="rId8"/>
     <sheet name="Int Reliability" sheetId="18" r:id="rId9"/>
     <sheet name="Non-Int Reliability" sheetId="19" r:id="rId10"/>
-    <sheet name="Scorecard_Safety" sheetId="21" r:id="rId11"/>
-    <sheet name="Scorecard_Infrastructure" sheetId="22" r:id="rId12"/>
-    <sheet name="Scorecard_Sys_Per_Reli" sheetId="23" r:id="rId13"/>
-    <sheet name="Scorecard_Transit_As_Man" sheetId="24" r:id="rId14"/>
-    <sheet name="Scorecard_Transit_Safety" sheetId="25" r:id="rId15"/>
-    <sheet name="FATALITIES COMP" sheetId="3" state="hidden" r:id="rId16"/>
+    <sheet name="UL_FRB" sheetId="26" r:id="rId11"/>
+    <sheet name="UL_CB" sheetId="27" r:id="rId12"/>
+    <sheet name="UL_SA" sheetId="28" r:id="rId13"/>
+    <sheet name="UL_ST" sheetId="29" r:id="rId14"/>
+    <sheet name="Scorecard_Safety" sheetId="21" r:id="rId15"/>
+    <sheet name="Scorecard_Infrastructure" sheetId="22" r:id="rId16"/>
+    <sheet name="Scorecard_Sys_Per_Reli" sheetId="23" r:id="rId17"/>
+    <sheet name="Scorecard_Transit_As_Man" sheetId="24" r:id="rId18"/>
+    <sheet name="Scorecard_Transit_Safety" sheetId="25" r:id="rId19"/>
+    <sheet name="FATALITIES COMP" sheetId="3" state="hidden" r:id="rId20"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -51,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="141">
   <si>
     <t>Alachua</t>
   </si>
@@ -471,6 +475,9 @@
   </si>
   <si>
     <t>Paratransit (Palm Tran Connection)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Percent Of Vehicles </t>
   </si>
 </sst>
 </file>
@@ -1192,6 +1199,427 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70545EE8-3393-48FF-8B94-A68F78870296}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="19.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2018</v>
+      </c>
+      <c r="B2" s="15">
+        <v>0</v>
+      </c>
+      <c r="C2" s="15">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2019</v>
+      </c>
+      <c r="B3" s="15">
+        <v>0.65</v>
+      </c>
+      <c r="C3" s="15">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2020</v>
+      </c>
+      <c r="B4" s="15">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="C4" s="15">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2021</v>
+      </c>
+      <c r="B5" s="15">
+        <v>0.15</v>
+      </c>
+      <c r="C5" s="15">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>2022</v>
+      </c>
+      <c r="B6" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C6" s="15">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2023</v>
+      </c>
+      <c r="B7" s="15">
+        <v>0.18</v>
+      </c>
+      <c r="C7" s="15">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>2024</v>
+      </c>
+      <c r="B8" s="15">
+        <v>0.19</v>
+      </c>
+      <c r="C8" s="15">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>2025</v>
+      </c>
+      <c r="B9" s="15">
+        <v>0.13</v>
+      </c>
+      <c r="C9" s="15">
+        <v>0.15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8768E2E-41F2-4128-AF4B-DB787856BFE5}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="19.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2018</v>
+      </c>
+      <c r="B2" s="15">
+        <v>0</v>
+      </c>
+      <c r="C2" s="15">
+        <v>0.1477</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2019</v>
+      </c>
+      <c r="B3" s="15">
+        <v>0.36</v>
+      </c>
+      <c r="C3" s="15">
+        <v>0.1477</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2020</v>
+      </c>
+      <c r="B4" s="15">
+        <v>0.21</v>
+      </c>
+      <c r="C4" s="15">
+        <v>0.1477</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2021</v>
+      </c>
+      <c r="B5" s="15">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="C5" s="15">
+        <v>0.1477</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>2022</v>
+      </c>
+      <c r="B6" s="15">
+        <v>0.09</v>
+      </c>
+      <c r="C6" s="15">
+        <v>0.1477</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2023</v>
+      </c>
+      <c r="B7" s="15">
+        <v>0.15</v>
+      </c>
+      <c r="C7" s="15">
+        <v>0.1477</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>2024</v>
+      </c>
+      <c r="B8" s="15">
+        <v>0.04</v>
+      </c>
+      <c r="C8" s="15">
+        <v>0.1477</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>2025</v>
+      </c>
+      <c r="B9" s="15">
+        <v>0.14799999999999999</v>
+      </c>
+      <c r="C9" s="15">
+        <v>0.1477</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47C9403F-1360-4C9E-9A0D-37F31FFD517C}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="19.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2018</v>
+      </c>
+      <c r="B2" s="15">
+        <v>0.26</v>
+      </c>
+      <c r="C2" s="15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2019</v>
+      </c>
+      <c r="B3" s="15">
+        <v>0.86</v>
+      </c>
+      <c r="C3" s="15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2020</v>
+      </c>
+      <c r="B4" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C4" s="15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2021</v>
+      </c>
+      <c r="B5" s="15">
+        <v>0.06</v>
+      </c>
+      <c r="C5" s="15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>2022</v>
+      </c>
+      <c r="B6" s="15">
+        <v>0.35</v>
+      </c>
+      <c r="C6" s="15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2023</v>
+      </c>
+      <c r="B7" s="15">
+        <v>0.17</v>
+      </c>
+      <c r="C7" s="15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>2024</v>
+      </c>
+      <c r="B8" s="15">
+        <v>0.43</v>
+      </c>
+      <c r="C8" s="15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>2025</v>
+      </c>
+      <c r="B9" s="15">
+        <v>0.69399999999999995</v>
+      </c>
+      <c r="C9" s="15">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F62C98EA-F049-4A45-95E1-AA425574422A}">
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="19.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2018</v>
+      </c>
+      <c r="B2" s="15">
+        <v>0.26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2019</v>
+      </c>
+      <c r="B3" s="15">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2020</v>
+      </c>
+      <c r="B4" s="15">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2021</v>
+      </c>
+      <c r="B5" s="15">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>2022</v>
+      </c>
+      <c r="B6" s="15">
+        <v>0.28000000000000003</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2023</v>
+      </c>
+      <c r="B7" s="15">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>2024</v>
+      </c>
+      <c r="B8" s="15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>2025</v>
+      </c>
+      <c r="B9" s="15">
+        <v>0.19700000000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B420F60-609B-4AA9-97E6-C695A4A591CA}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1289,7 +1717,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B84F7EA7-DBFB-4CBA-A1A1-E112D361DAFF}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1422,7 +1850,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8FF0919-3905-4425-81BF-3149EAA458D8}">
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1493,7 +1921,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1963ABED-C249-4004-B31E-6E99DC2E6917}">
   <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1697,7 +2125,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C3051EB-9F2E-4379-8AFD-5E4458A288D3}">
   <dimension ref="A1:E15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1969,7 +2397,105 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{504C1906-E774-4362-B18C-74A3CE45CFF8}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="14.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2018</v>
+      </c>
+      <c r="B2" s="9">
+        <v>1194</v>
+      </c>
+      <c r="C2" s="8">
+        <v>8.42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2019</v>
+      </c>
+      <c r="B3" s="9">
+        <v>1020</v>
+      </c>
+      <c r="C3" s="8">
+        <v>7.08</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2020</v>
+      </c>
+      <c r="B4" s="10">
+        <v>916</v>
+      </c>
+      <c r="C4" s="8">
+        <v>6.91</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2021</v>
+      </c>
+      <c r="B5" s="10">
+        <v>890</v>
+      </c>
+      <c r="C5" s="8">
+        <v>6.45</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>2022</v>
+      </c>
+      <c r="B6" s="10">
+        <v>818</v>
+      </c>
+      <c r="C6" s="8">
+        <v>5.73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2023</v>
+      </c>
+      <c r="B7" s="10">
+        <v>766</v>
+      </c>
+      <c r="C7" s="8">
+        <v>5.16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>2024</v>
+      </c>
+      <c r="B8" s="7">
+        <v>683</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DE6782D-92DC-4DC3-BB49-53C081EF8C06}">
   <dimension ref="A1:BP8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3495,104 +4021,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{504C1906-E774-4362-B18C-74A3CE45CFF8}">
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="14.5703125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B1" t="s">
-        <v>69</v>
-      </c>
-      <c r="C1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>2018</v>
-      </c>
-      <c r="B2" s="9">
-        <v>1194</v>
-      </c>
-      <c r="C2" s="8">
-        <v>8.42</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2019</v>
-      </c>
-      <c r="B3" s="9">
-        <v>1020</v>
-      </c>
-      <c r="C3" s="8">
-        <v>7.08</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>2020</v>
-      </c>
-      <c r="B4" s="10">
-        <v>916</v>
-      </c>
-      <c r="C4" s="8">
-        <v>6.91</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>2021</v>
-      </c>
-      <c r="B5" s="10">
-        <v>890</v>
-      </c>
-      <c r="C5" s="8">
-        <v>6.45</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>2022</v>
-      </c>
-      <c r="B6" s="10">
-        <v>818</v>
-      </c>
-      <c r="C6" s="8">
-        <v>5.73</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>2023</v>
-      </c>
-      <c r="B7" s="10">
-        <v>766</v>
-      </c>
-      <c r="C7" s="8">
-        <v>5.16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>2024</v>
-      </c>
-      <c r="B8" s="7">
-        <v>683</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{881ACF1F-DA10-4F3C-BBFE-3F6465156627}">
   <dimension ref="A1:C8"/>

</xml_diff>

<commit_message>
Restore dashboard header and styling after title alignment troubleshooting
</commit_message>
<xml_diff>
--- a/Performance_Measures_R.xlsx
+++ b/Performance_Measures_R.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://palmbeachtpa-my.sharepoint.com/personal/skan_palmbeachmpo_org/Documents/Documents/Performance_Measures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="400" documentId="8_{6E25A293-DAE1-403C-87C6-760DEF9E0950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E778E3EC-2CAB-4D41-8F8F-DF2C02C5FE69}"/>
+  <xr:revisionPtr revIDLastSave="484" documentId="8_{6E25A293-DAE1-403C-87C6-760DEF9E0950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA6E3AAA-D7EF-4859-92B5-60CA846D4F6E}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="13" xr2:uid="{47865025-DE32-4D87-A21F-3C532F9D4B3D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="20" activeTab="23" xr2:uid="{47865025-DE32-4D87-A21F-3C532F9D4B3D}"/>
   </bookViews>
   <sheets>
     <sheet name="FATALITIES" sheetId="7" r:id="rId1"/>
@@ -27,12 +27,17 @@
     <sheet name="UL_CB" sheetId="27" r:id="rId12"/>
     <sheet name="UL_SA" sheetId="28" r:id="rId13"/>
     <sheet name="UL_ST" sheetId="29" r:id="rId14"/>
-    <sheet name="Scorecard_Safety" sheetId="21" r:id="rId15"/>
-    <sheet name="Scorecard_Infrastructure" sheetId="22" r:id="rId16"/>
-    <sheet name="Scorecard_Sys_Per_Reli" sheetId="23" r:id="rId17"/>
-    <sheet name="Scorecard_Transit_As_Man" sheetId="24" r:id="rId18"/>
-    <sheet name="Scorecard_Transit_Safety" sheetId="25" r:id="rId19"/>
-    <sheet name="FATALITIES COMP" sheetId="3" state="hidden" r:id="rId20"/>
+    <sheet name="Trirail_Loco" sheetId="30" r:id="rId15"/>
+    <sheet name="Trirail_PER_R" sheetId="31" r:id="rId16"/>
+    <sheet name="Trirail_Sup_Main" sheetId="32" r:id="rId17"/>
+    <sheet name="PT_Safety_SC" sheetId="34" r:id="rId18"/>
+    <sheet name="Trirail_Facilties" sheetId="33" r:id="rId19"/>
+    <sheet name="Scorecard_Safety" sheetId="21" r:id="rId20"/>
+    <sheet name="Scorecard_Infrastructure" sheetId="22" r:id="rId21"/>
+    <sheet name="Scorecard_Sys_Per_Reli" sheetId="23" r:id="rId22"/>
+    <sheet name="Scorecard_Transit_As_Man" sheetId="24" r:id="rId23"/>
+    <sheet name="Scorecard_Transit_Safety" sheetId="25" r:id="rId24"/>
+    <sheet name="FATALITIES COMP" sheetId="3" state="hidden" r:id="rId25"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -55,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="143">
   <si>
     <t>Alachua</t>
   </si>
@@ -478,6 +483,12 @@
   </si>
   <si>
     <t xml:space="preserve">Percent Of Vehicles </t>
+  </si>
+  <si>
+    <t>Actual 2025</t>
+  </si>
+  <si>
+    <t>Target 2026</t>
   </si>
 </sst>
 </file>
@@ -581,7 +592,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -625,6 +636,10 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -983,12 +998,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFAE9F3B-BA9E-497C-8DE5-DBDC8EE87CC9}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="18.85546875" customWidth="1"/>
+    <col min="2" max="2" width="18.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>68</v>
       </c>
@@ -999,7 +1014,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2018</v>
       </c>
@@ -1010,7 +1025,7 @@
         <v>1.29</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2019</v>
       </c>
@@ -1021,7 +1036,7 @@
         <v>1.21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2020</v>
       </c>
@@ -1032,7 +1047,7 @@
         <v>1.4</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2021</v>
       </c>
@@ -1043,7 +1058,7 @@
         <v>1.56</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2022</v>
       </c>
@@ -1054,7 +1069,7 @@
         <v>1.63</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2023</v>
       </c>
@@ -1065,7 +1080,7 @@
         <v>1.22</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2024</v>
       </c>
@@ -1084,12 +1099,12 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CB9C645-8F86-45BC-BA51-DC3AF3602CC7}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="13.28515625" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>68</v>
       </c>
@@ -1100,7 +1115,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2017</v>
       </c>
@@ -1111,7 +1126,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2018</v>
       </c>
@@ -1122,7 +1137,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2019</v>
       </c>
@@ -1133,7 +1148,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2020</v>
       </c>
@@ -1144,7 +1159,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2021</v>
       </c>
@@ -1155,7 +1170,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2022</v>
       </c>
@@ -1166,7 +1181,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2023</v>
       </c>
@@ -1177,7 +1192,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2024</v>
       </c>
@@ -1201,12 +1216,12 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70545EE8-3393-48FF-8B94-A68F78870296}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="19.5703125" customWidth="1"/>
+    <col min="2" max="2" width="19.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>68</v>
       </c>
@@ -1217,7 +1232,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2018</v>
       </c>
@@ -1228,7 +1243,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2019</v>
       </c>
@@ -1239,7 +1254,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2020</v>
       </c>
@@ -1250,7 +1265,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2021</v>
       </c>
@@ -1261,7 +1276,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2022</v>
       </c>
@@ -1272,7 +1287,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2023</v>
       </c>
@@ -1283,7 +1298,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2024</v>
       </c>
@@ -1294,7 +1309,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2025</v>
       </c>
@@ -1313,12 +1328,12 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8768E2E-41F2-4128-AF4B-DB787856BFE5}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="19.5703125" customWidth="1"/>
+    <col min="2" max="2" width="19.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>68</v>
       </c>
@@ -1329,7 +1344,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2018</v>
       </c>
@@ -1340,7 +1355,7 @@
         <v>0.1477</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2019</v>
       </c>
@@ -1351,7 +1366,7 @@
         <v>0.1477</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2020</v>
       </c>
@@ -1362,7 +1377,7 @@
         <v>0.1477</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2021</v>
       </c>
@@ -1373,7 +1388,7 @@
         <v>0.1477</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2022</v>
       </c>
@@ -1384,7 +1399,7 @@
         <v>0.1477</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2023</v>
       </c>
@@ -1395,7 +1410,7 @@
         <v>0.1477</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2024</v>
       </c>
@@ -1406,7 +1421,7 @@
         <v>0.1477</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2025</v>
       </c>
@@ -1425,12 +1440,12 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47C9403F-1360-4C9E-9A0D-37F31FFD517C}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="19.5703125" customWidth="1"/>
+    <col min="2" max="2" width="19.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>68</v>
       </c>
@@ -1441,7 +1456,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2018</v>
       </c>
@@ -1452,7 +1467,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2019</v>
       </c>
@@ -1463,7 +1478,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2020</v>
       </c>
@@ -1474,7 +1489,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2021</v>
       </c>
@@ -1485,7 +1500,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2022</v>
       </c>
@@ -1496,7 +1511,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2023</v>
       </c>
@@ -1507,7 +1522,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2024</v>
       </c>
@@ -1518,7 +1533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2025</v>
       </c>
@@ -1537,12 +1552,12 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F62C98EA-F049-4A45-95E1-AA425574422A}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="19.5703125" customWidth="1"/>
+    <col min="2" max="2" width="19.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>68</v>
       </c>
@@ -1550,7 +1565,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2018</v>
       </c>
@@ -1558,7 +1573,7 @@
         <v>0.26</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2019</v>
       </c>
@@ -1566,7 +1581,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2020</v>
       </c>
@@ -1574,7 +1589,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2021</v>
       </c>
@@ -1582,7 +1597,7 @@
         <v>0.17</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2022</v>
       </c>
@@ -1590,7 +1605,7 @@
         <v>0.28000000000000003</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2023</v>
       </c>
@@ -1598,7 +1613,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2024</v>
       </c>
@@ -1606,7 +1621,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2025</v>
       </c>
@@ -1620,96 +1635,88 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B420F60-609B-4AA9-97E6-C695A4A591CA}">
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDBE33F8-F6FD-46D3-B669-CD9D8BFF9D18}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="43" customWidth="1"/>
-    <col min="3" max="3" width="15.85546875" customWidth="1"/>
+    <col min="2" max="2" width="19.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="B1" t="s">
-        <v>89</v>
+        <v>140</v>
       </c>
       <c r="C1" t="s">
-        <v>88</v>
-      </c>
-      <c r="D1" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C2">
-        <v>207.4</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>87</v>
-      </c>
-      <c r="B3" t="s">
-        <v>83</v>
-      </c>
-      <c r="C3">
-        <v>1.45</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>86</v>
-      </c>
-      <c r="B4" t="s">
-        <v>83</v>
-      </c>
-      <c r="C4">
-        <v>812.2</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>85</v>
-      </c>
-      <c r="B5" t="s">
-        <v>83</v>
-      </c>
-      <c r="C5">
-        <v>5.73</v>
-      </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>84</v>
-      </c>
-      <c r="B6" t="s">
-        <v>83</v>
-      </c>
-      <c r="C6">
-        <v>203.8</v>
-      </c>
-      <c r="D6">
-        <v>0</v>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>2019</v>
+      </c>
+      <c r="B2" s="23">
+        <v>0.25</v>
+      </c>
+      <c r="C2" s="15">
+        <v>0.28599999999999998</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2020</v>
+      </c>
+      <c r="B3" s="23">
+        <v>0.26700000000000002</v>
+      </c>
+      <c r="C3" s="15">
+        <v>0.28599999999999998</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>2021</v>
+      </c>
+      <c r="B4" s="23">
+        <v>0.26300000000000001</v>
+      </c>
+      <c r="C4" s="15">
+        <v>0.28599999999999998</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>2022</v>
+      </c>
+      <c r="B5" s="23">
+        <v>0.3</v>
+      </c>
+      <c r="C5" s="15">
+        <v>0.28599999999999998</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>2023</v>
+      </c>
+      <c r="B6" s="23">
+        <v>0.32</v>
+      </c>
+      <c r="C6" s="15">
+        <v>0.28599999999999998</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>2024</v>
+      </c>
+      <c r="B7" s="23">
+        <v>0.25</v>
+      </c>
+      <c r="C7" s="15">
+        <v>0.28599999999999998</v>
       </c>
     </row>
   </sheetData>
@@ -1718,131 +1725,96 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B84F7EA7-DBFB-4CBA-A1A1-E112D361DAFF}">
-  <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="43" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2012453B-2FD9-4676-A93F-5D42E7C311A7}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>92</v>
+        <v>68</v>
       </c>
       <c r="B1" t="s">
-        <v>90</v>
+        <v>140</v>
       </c>
       <c r="C1" t="s">
-        <v>89</v>
-      </c>
-      <c r="D1" t="s">
-        <v>93</v>
-      </c>
-      <c r="E1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>91</v>
-      </c>
-      <c r="B2" t="s">
-        <v>95</v>
-      </c>
-      <c r="C2" t="s">
-        <v>96</v>
-      </c>
-      <c r="D2" s="20">
-        <v>0.83199999999999996</v>
-      </c>
-      <c r="E2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>91</v>
-      </c>
-      <c r="B3" t="s">
-        <v>98</v>
-      </c>
-      <c r="C3" t="s">
-        <v>96</v>
-      </c>
-      <c r="D3" s="20">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>2018</v>
+      </c>
+      <c r="B2" s="15">
+        <v>0.08</v>
+      </c>
+      <c r="C2" s="15">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2019</v>
+      </c>
+      <c r="B3" s="23">
+        <v>3.3000000000000002E-2</v>
+      </c>
+      <c r="C3" s="15">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>2020</v>
+      </c>
+      <c r="B4" s="23">
         <v>0</v>
       </c>
-      <c r="E3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>100</v>
-      </c>
-      <c r="B4" t="s">
-        <v>101</v>
-      </c>
-      <c r="C4" t="s">
-        <v>83</v>
-      </c>
-      <c r="D4" s="20">
-        <v>0.54700000000000004</v>
-      </c>
-      <c r="E4" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>100</v>
-      </c>
-      <c r="B5" t="s">
-        <v>103</v>
-      </c>
-      <c r="C5" t="s">
-        <v>96</v>
-      </c>
-      <c r="D5" s="20">
-        <v>0</v>
-      </c>
-      <c r="E5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>100</v>
-      </c>
-      <c r="B6" t="s">
-        <v>104</v>
-      </c>
-      <c r="C6" t="s">
-        <v>96</v>
-      </c>
-      <c r="D6" s="20">
-        <v>0.56299999999999994</v>
-      </c>
-      <c r="E6" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>100</v>
-      </c>
-      <c r="B7" t="s">
-        <v>106</v>
-      </c>
-      <c r="C7" t="s">
-        <v>96</v>
-      </c>
-      <c r="D7" s="20">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="E7" t="s">
-        <v>99</v>
+      <c r="C4" s="15">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>2021</v>
+      </c>
+      <c r="B5" s="23">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="C5" s="15">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>2022</v>
+      </c>
+      <c r="B6" s="23">
+        <v>1.5E-3</v>
+      </c>
+      <c r="C6" s="15">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>2023</v>
+      </c>
+      <c r="B7" s="23">
+        <v>1.6000000000000001E-3</v>
+      </c>
+      <c r="C7" s="15">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>2024</v>
+      </c>
+      <c r="B8" s="23">
+        <v>1.6000000000000001E-3</v>
+      </c>
+      <c r="C8" s="15">
+        <v>0.03</v>
       </c>
     </row>
   </sheetData>
@@ -1851,69 +1823,85 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8FF0919-3905-4425-81BF-3149EAA458D8}">
-  <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="56.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBB831B4-CACE-4DDE-9F5D-2A702D15F4A9}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="B1" t="s">
-        <v>89</v>
+        <v>140</v>
       </c>
       <c r="C1" t="s">
-        <v>93</v>
-      </c>
-      <c r="D1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>107</v>
-      </c>
-      <c r="B2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C2" s="21">
-        <v>0.623</v>
-      </c>
-      <c r="D2" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>109</v>
-      </c>
-      <c r="B3" t="s">
-        <v>96</v>
-      </c>
-      <c r="C3" s="21">
-        <v>0.86799999999999999</v>
-      </c>
-      <c r="D3" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>110</v>
-      </c>
-      <c r="B4" t="s">
-        <v>83</v>
-      </c>
-      <c r="C4">
-        <v>2.09</v>
-      </c>
-      <c r="D4" t="s">
-        <v>111</v>
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>2019</v>
+      </c>
+      <c r="B2" s="23">
+        <v>0.222</v>
+      </c>
+      <c r="C2" s="15">
+        <v>0.41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2020</v>
+      </c>
+      <c r="B3" s="23">
+        <v>0.44400000000000001</v>
+      </c>
+      <c r="C3" s="15">
+        <v>0.41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>2021</v>
+      </c>
+      <c r="B4" s="23">
+        <v>0.5</v>
+      </c>
+      <c r="C4" s="15">
+        <v>0.41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>2022</v>
+      </c>
+      <c r="B5" s="23">
+        <v>0.625</v>
+      </c>
+      <c r="C5" s="15">
+        <v>0.41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>2023</v>
+      </c>
+      <c r="B6" s="23">
+        <v>0.41</v>
+      </c>
+      <c r="C6" s="15">
+        <v>0.41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>2024</v>
+      </c>
+      <c r="B7" s="23">
+        <v>0.25</v>
+      </c>
+      <c r="C7" s="15">
+        <v>0.41</v>
       </c>
     </row>
   </sheetData>
@@ -1922,18 +1910,17 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1963ABED-C249-4004-B31E-6E99DC2E6917}">
-  <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF8158D5-45CD-485F-9E37-C77E69A730F0}">
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="64.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>92</v>
       </c>
@@ -1941,455 +1928,284 @@
         <v>90</v>
       </c>
       <c r="C1" t="s">
-        <v>112</v>
+        <v>141</v>
       </c>
       <c r="D1" t="s">
-        <v>113</v>
-      </c>
-      <c r="E1" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>115</v>
+        <v>142</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="24" t="s">
+        <v>132</v>
       </c>
       <c r="B2" t="s">
-        <v>116</v>
-      </c>
-      <c r="C2" t="s">
-        <v>96</v>
-      </c>
-      <c r="D2" s="15">
+        <v>71</v>
+      </c>
+      <c r="C2">
         <v>0</v>
       </c>
-      <c r="E2" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>115</v>
-      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="24"/>
       <c r="B3" t="s">
-        <v>118</v>
-      </c>
-      <c r="C3" t="s">
-        <v>96</v>
-      </c>
-      <c r="D3" s="15">
+        <v>134</v>
+      </c>
+      <c r="C3">
+        <v>0.01</v>
+      </c>
+      <c r="D3">
         <v>0</v>
       </c>
-      <c r="E3" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>115</v>
-      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="24"/>
       <c r="B4" t="s">
-        <v>119</v>
-      </c>
-      <c r="C4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D4" s="15">
+        <v>72</v>
+      </c>
+      <c r="C4">
+        <v>44</v>
+      </c>
+      <c r="D4">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="24"/>
+      <c r="B5" t="s">
+        <v>135</v>
+      </c>
+      <c r="C5">
+        <v>0.1</v>
+      </c>
+      <c r="D5">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="24"/>
+      <c r="B6" t="s">
+        <v>136</v>
+      </c>
+      <c r="C6">
+        <v>49</v>
+      </c>
+      <c r="D6">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="24"/>
+      <c r="B7" t="s">
+        <v>137</v>
+      </c>
+      <c r="C7">
+        <v>0.6</v>
+      </c>
+      <c r="D7">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="24"/>
+      <c r="B8" t="s">
+        <v>138</v>
+      </c>
+      <c r="C8" s="22">
+        <v>7929</v>
+      </c>
+      <c r="D8" s="22">
+        <v>14000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="24" t="s">
+        <v>139</v>
+      </c>
+      <c r="B9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C9">
         <v>0</v>
       </c>
-      <c r="E4" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>115</v>
-      </c>
-      <c r="B5" t="s">
-        <v>120</v>
-      </c>
-      <c r="C5" t="s">
-        <v>83</v>
-      </c>
-      <c r="D5" s="21">
-        <v>0.434</v>
-      </c>
-      <c r="E5" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>115</v>
-      </c>
-      <c r="B6" t="s">
-        <v>121</v>
-      </c>
-      <c r="C6" t="s">
-        <v>96</v>
-      </c>
-      <c r="D6" s="21">
-        <v>5.0000000000000001E-4</v>
-      </c>
-      <c r="E6" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>115</v>
-      </c>
-      <c r="B7" t="s">
-        <v>122</v>
-      </c>
-      <c r="C7" t="s">
-        <v>96</v>
-      </c>
-      <c r="D7" s="15">
+      <c r="D9">
         <v>0</v>
       </c>
-      <c r="E7" s="15">
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="24"/>
+      <c r="B10" t="s">
+        <v>134</v>
+      </c>
+      <c r="C10">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>123</v>
-      </c>
-      <c r="B8" t="s">
-        <v>124</v>
-      </c>
-      <c r="C8" t="s">
-        <v>83</v>
-      </c>
-      <c r="D8" s="15">
-        <v>0.32</v>
-      </c>
-      <c r="E8" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>123</v>
-      </c>
-      <c r="B9" t="s">
-        <v>126</v>
-      </c>
-      <c r="C9" t="s">
-        <v>96</v>
-      </c>
-      <c r="D9" s="15">
-        <v>0.41</v>
-      </c>
-      <c r="E9" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>123</v>
-      </c>
-      <c r="B10" t="s">
-        <v>128</v>
-      </c>
-      <c r="C10" t="s">
-        <v>96</v>
-      </c>
-      <c r="D10" s="15">
+      <c r="D10">
         <v>0</v>
       </c>
-      <c r="E10" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>123</v>
-      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="24"/>
       <c r="B11" t="s">
-        <v>130</v>
-      </c>
-      <c r="C11" t="s">
-        <v>96</v>
-      </c>
-      <c r="D11" s="21">
-        <v>1.6000000000000001E-3</v>
-      </c>
-      <c r="E11" t="s">
-        <v>131</v>
+        <v>72</v>
+      </c>
+      <c r="C11">
+        <v>17</v>
+      </c>
+      <c r="D11">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="24"/>
+      <c r="B12" t="s">
+        <v>135</v>
+      </c>
+      <c r="C12">
+        <v>0.2</v>
+      </c>
+      <c r="D12">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="24"/>
+      <c r="B13" t="s">
+        <v>136</v>
+      </c>
+      <c r="C13">
+        <v>17</v>
+      </c>
+      <c r="D13">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="24"/>
+      <c r="B14" t="s">
+        <v>137</v>
+      </c>
+      <c r="C14">
+        <v>0.2</v>
+      </c>
+      <c r="D14">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="24"/>
+      <c r="B15" t="s">
+        <v>138</v>
+      </c>
+      <c r="C15" s="22">
+        <v>15101</v>
+      </c>
+      <c r="D15" s="22">
+        <v>7700</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:A8"/>
+    <mergeCell ref="A9:A15"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C3051EB-9F2E-4379-8AFD-5E4458A288D3}">
-  <dimension ref="A1:E15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="32.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.28515625" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8A2B925-F3EE-472B-B53C-CA468800D579}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>92</v>
+        <v>68</v>
       </c>
       <c r="B1" t="s">
-        <v>90</v>
+        <v>140</v>
       </c>
       <c r="C1" t="s">
-        <v>112</v>
-      </c>
-      <c r="D1" t="s">
-        <v>93</v>
-      </c>
-      <c r="E1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>132</v>
-      </c>
-      <c r="B2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C2" t="s">
-        <v>133</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>2018</v>
+      </c>
+      <c r="B2" s="15">
+        <v>0.3</v>
+      </c>
+      <c r="C2" s="15">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2019</v>
+      </c>
+      <c r="B3" s="23">
+        <v>0.05</v>
+      </c>
+      <c r="C3" s="15">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>2020</v>
+      </c>
+      <c r="B4" s="23">
+        <v>0.05</v>
+      </c>
+      <c r="C4" s="15">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>2021</v>
+      </c>
+      <c r="B5" s="23">
+        <v>0.05</v>
+      </c>
+      <c r="C5" s="15">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>2022</v>
+      </c>
+      <c r="B6" s="23">
+        <v>0.33</v>
+      </c>
+      <c r="C6" s="15">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>2023</v>
+      </c>
+      <c r="B7" s="23">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>132</v>
-      </c>
-      <c r="B3" t="s">
-        <v>134</v>
-      </c>
-      <c r="C3" t="s">
-        <v>133</v>
-      </c>
-      <c r="D3">
-        <v>0.01</v>
-      </c>
-      <c r="E3">
+      <c r="C7" s="15">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>2024</v>
+      </c>
+      <c r="B8" s="23">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>132</v>
-      </c>
-      <c r="B4" t="s">
-        <v>72</v>
-      </c>
-      <c r="C4" t="s">
-        <v>133</v>
-      </c>
-      <c r="D4">
-        <v>18</v>
-      </c>
-      <c r="E4">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>132</v>
-      </c>
-      <c r="B5" t="s">
-        <v>135</v>
-      </c>
-      <c r="C5" t="s">
-        <v>133</v>
-      </c>
-      <c r="D5">
-        <v>0.2</v>
-      </c>
-      <c r="E5">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>132</v>
-      </c>
-      <c r="B6" t="s">
-        <v>136</v>
-      </c>
-      <c r="C6" t="s">
-        <v>133</v>
-      </c>
-      <c r="D6">
-        <v>49</v>
-      </c>
-      <c r="E6">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>132</v>
-      </c>
-      <c r="B7" t="s">
-        <v>137</v>
-      </c>
-      <c r="C7" t="s">
-        <v>133</v>
-      </c>
-      <c r="D7">
-        <v>0.7</v>
-      </c>
-      <c r="E7">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>132</v>
-      </c>
-      <c r="B8" t="s">
-        <v>138</v>
-      </c>
-      <c r="C8" t="s">
-        <v>133</v>
-      </c>
-      <c r="D8" s="22">
-        <v>6609</v>
-      </c>
-      <c r="E8" s="22">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>139</v>
-      </c>
-      <c r="B9" t="s">
-        <v>71</v>
-      </c>
-      <c r="C9" t="s">
-        <v>133</v>
-      </c>
-      <c r="D9">
-        <v>0</v>
-      </c>
-      <c r="E9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>139</v>
-      </c>
-      <c r="B10" t="s">
-        <v>134</v>
-      </c>
-      <c r="C10" t="s">
-        <v>133</v>
-      </c>
-      <c r="D10">
-        <v>0</v>
-      </c>
-      <c r="E10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>139</v>
-      </c>
-      <c r="B11" t="s">
-        <v>72</v>
-      </c>
-      <c r="C11" t="s">
-        <v>133</v>
-      </c>
-      <c r="D11">
-        <v>20</v>
-      </c>
-      <c r="E11">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>139</v>
-      </c>
-      <c r="B12" t="s">
-        <v>135</v>
-      </c>
-      <c r="C12" t="s">
-        <v>133</v>
-      </c>
-      <c r="D12">
-        <v>0.2</v>
-      </c>
-      <c r="E12">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>139</v>
-      </c>
-      <c r="B13" t="s">
-        <v>136</v>
-      </c>
-      <c r="C13" t="s">
-        <v>133</v>
-      </c>
-      <c r="D13">
-        <v>14</v>
-      </c>
-      <c r="E13">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>139</v>
-      </c>
-      <c r="B14" t="s">
-        <v>137</v>
-      </c>
-      <c r="C14" t="s">
-        <v>133</v>
-      </c>
-      <c r="D14">
-        <v>0.1</v>
-      </c>
-      <c r="E14">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>139</v>
-      </c>
-      <c r="B15" t="s">
-        <v>138</v>
-      </c>
-      <c r="C15" t="s">
-        <v>133</v>
-      </c>
-      <c r="D15" s="22">
-        <v>10569</v>
-      </c>
-      <c r="E15" s="22">
-        <v>7700</v>
+      <c r="C8" s="15">
+        <v>0.05</v>
       </c>
     </row>
   </sheetData>
@@ -2400,12 +2216,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{504C1906-E774-4362-B18C-74A3CE45CFF8}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="14.5703125" customWidth="1"/>
+    <col min="2" max="2" width="14.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>68</v>
       </c>
@@ -2416,7 +2232,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2018</v>
       </c>
@@ -2427,7 +2243,7 @@
         <v>8.42</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2019</v>
       </c>
@@ -2438,7 +2254,7 @@
         <v>7.08</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2020</v>
       </c>
@@ -2449,7 +2265,7 @@
         <v>6.91</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2021</v>
       </c>
@@ -2460,7 +2276,7 @@
         <v>6.45</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2022</v>
       </c>
@@ -2471,7 +2287,7 @@
         <v>5.73</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2023</v>
       </c>
@@ -2482,7 +2298,7 @@
         <v>5.16</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2024</v>
       </c>
@@ -2496,11 +2312,753 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B420F60-609B-4AA9-97E6-C695A4A591CA}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="43" customWidth="1"/>
+    <col min="3" max="3" width="15.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2">
+        <v>207.4</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C3">
+        <v>1.45</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4">
+        <v>812.2</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C5">
+        <v>5.73</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6">
+        <v>203.8</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B84F7EA7-DBFB-4CBA-A1A1-E112D361DAFF}">
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="43" customWidth="1"/>
+    <col min="4" max="4" width="15.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="24" t="s">
+        <v>91</v>
+      </c>
+      <c r="B2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D2" s="20">
+        <v>0.83199999999999996</v>
+      </c>
+      <c r="E2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="24"/>
+      <c r="B3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C3" t="s">
+        <v>96</v>
+      </c>
+      <c r="D3" s="20">
+        <v>0</v>
+      </c>
+      <c r="E3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="24" t="s">
+        <v>100</v>
+      </c>
+      <c r="B4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C4" t="s">
+        <v>83</v>
+      </c>
+      <c r="D4" s="20">
+        <v>0.54700000000000004</v>
+      </c>
+      <c r="E4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="24"/>
+      <c r="B5" t="s">
+        <v>103</v>
+      </c>
+      <c r="C5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D5" s="20">
+        <v>0</v>
+      </c>
+      <c r="E5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="24"/>
+      <c r="B6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C6" t="s">
+        <v>96</v>
+      </c>
+      <c r="D6" s="20">
+        <v>0.56299999999999994</v>
+      </c>
+      <c r="E6" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="24"/>
+      <c r="B7" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7" t="s">
+        <v>96</v>
+      </c>
+      <c r="D7" s="20">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="E7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A4:A7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8FF0919-3905-4425-81BF-3149EAA458D8}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="56.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2" s="21">
+        <v>0.623</v>
+      </c>
+      <c r="D2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C3" s="21">
+        <v>0.86799999999999999</v>
+      </c>
+      <c r="D3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4">
+        <v>2.09</v>
+      </c>
+      <c r="D4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1963ABED-C249-4004-B31E-6E99DC2E6917}">
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="64.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="24" t="s">
+        <v>115</v>
+      </c>
+      <c r="B2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D2" s="15">
+        <v>0</v>
+      </c>
+      <c r="E2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="24"/>
+      <c r="B3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C3" t="s">
+        <v>96</v>
+      </c>
+      <c r="D3" s="15">
+        <v>0</v>
+      </c>
+      <c r="E3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="24"/>
+      <c r="B4" t="s">
+        <v>119</v>
+      </c>
+      <c r="C4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D4" s="15">
+        <v>0</v>
+      </c>
+      <c r="E4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="24"/>
+      <c r="B5" t="s">
+        <v>120</v>
+      </c>
+      <c r="C5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D5" s="21">
+        <v>0.434</v>
+      </c>
+      <c r="E5" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="24"/>
+      <c r="B6" t="s">
+        <v>121</v>
+      </c>
+      <c r="C6" t="s">
+        <v>96</v>
+      </c>
+      <c r="D6" s="21">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="E6" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="24"/>
+      <c r="B7" t="s">
+        <v>122</v>
+      </c>
+      <c r="C7" t="s">
+        <v>96</v>
+      </c>
+      <c r="D7" s="15">
+        <v>0</v>
+      </c>
+      <c r="E7" s="15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="24" t="s">
+        <v>123</v>
+      </c>
+      <c r="B8" t="s">
+        <v>124</v>
+      </c>
+      <c r="C8" t="s">
+        <v>83</v>
+      </c>
+      <c r="D8" s="15">
+        <v>0.32</v>
+      </c>
+      <c r="E8" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="24"/>
+      <c r="B9" t="s">
+        <v>126</v>
+      </c>
+      <c r="C9" t="s">
+        <v>96</v>
+      </c>
+      <c r="D9" s="15">
+        <v>0.41</v>
+      </c>
+      <c r="E9" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="24"/>
+      <c r="B10" t="s">
+        <v>128</v>
+      </c>
+      <c r="C10" t="s">
+        <v>96</v>
+      </c>
+      <c r="D10" s="15">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="24"/>
+      <c r="B11" t="s">
+        <v>130</v>
+      </c>
+      <c r="C11" t="s">
+        <v>96</v>
+      </c>
+      <c r="D11" s="21">
+        <v>1.6000000000000001E-3</v>
+      </c>
+      <c r="E11" t="s">
+        <v>131</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:A7"/>
+    <mergeCell ref="A8:A11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C3051EB-9F2E-4379-8AFD-5E4458A288D3}">
+  <dimension ref="A1:E15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="32.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="24" t="s">
+        <v>132</v>
+      </c>
+      <c r="B2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="24"/>
+      <c r="B3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C3" t="s">
+        <v>133</v>
+      </c>
+      <c r="D3">
+        <v>0.01</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="24"/>
+      <c r="B4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4" t="s">
+        <v>133</v>
+      </c>
+      <c r="D4">
+        <v>18</v>
+      </c>
+      <c r="E4">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="24"/>
+      <c r="B5" t="s">
+        <v>135</v>
+      </c>
+      <c r="C5" t="s">
+        <v>133</v>
+      </c>
+      <c r="D5">
+        <v>0.2</v>
+      </c>
+      <c r="E5">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="24"/>
+      <c r="B6" t="s">
+        <v>136</v>
+      </c>
+      <c r="C6" t="s">
+        <v>133</v>
+      </c>
+      <c r="D6">
+        <v>49</v>
+      </c>
+      <c r="E6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="24"/>
+      <c r="B7" t="s">
+        <v>137</v>
+      </c>
+      <c r="C7" t="s">
+        <v>133</v>
+      </c>
+      <c r="D7">
+        <v>0.7</v>
+      </c>
+      <c r="E7">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="24"/>
+      <c r="B8" t="s">
+        <v>138</v>
+      </c>
+      <c r="C8" t="s">
+        <v>133</v>
+      </c>
+      <c r="D8" s="22">
+        <v>6609</v>
+      </c>
+      <c r="E8" s="22">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="24" t="s">
+        <v>139</v>
+      </c>
+      <c r="B9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C9" t="s">
+        <v>133</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="24"/>
+      <c r="B10" t="s">
+        <v>134</v>
+      </c>
+      <c r="C10" t="s">
+        <v>133</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="24"/>
+      <c r="B11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C11" t="s">
+        <v>133</v>
+      </c>
+      <c r="D11">
+        <v>20</v>
+      </c>
+      <c r="E11">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="24"/>
+      <c r="B12" t="s">
+        <v>135</v>
+      </c>
+      <c r="C12" t="s">
+        <v>133</v>
+      </c>
+      <c r="D12">
+        <v>0.2</v>
+      </c>
+      <c r="E12">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="24"/>
+      <c r="B13" t="s">
+        <v>136</v>
+      </c>
+      <c r="C13" t="s">
+        <v>133</v>
+      </c>
+      <c r="D13">
+        <v>14</v>
+      </c>
+      <c r="E13">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="24"/>
+      <c r="B14" t="s">
+        <v>137</v>
+      </c>
+      <c r="C14" t="s">
+        <v>133</v>
+      </c>
+      <c r="D14">
+        <v>0.1</v>
+      </c>
+      <c r="E14">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="24"/>
+      <c r="B15" t="s">
+        <v>138</v>
+      </c>
+      <c r="C15" t="s">
+        <v>133</v>
+      </c>
+      <c r="D15" s="22">
+        <v>10569</v>
+      </c>
+      <c r="E15" s="22">
+        <v>7700</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:A8"/>
+    <mergeCell ref="A9:A15"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DE6782D-92DC-4DC3-BB49-53C081EF8C06}">
   <dimension ref="A1:BP8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:68" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -2706,7 +3264,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="2" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:68" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2018</v>
       </c>
@@ -2912,7 +3470,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:68" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2019</v>
       </c>
@@ -3118,7 +3676,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:68" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2020</v>
       </c>
@@ -3324,7 +3882,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:68" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2021</v>
       </c>
@@ -3530,7 +4088,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:68" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2022</v>
       </c>
@@ -3736,7 +4294,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:68" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2023</v>
       </c>
@@ -3942,7 +4500,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:68" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2024</v>
       </c>
@@ -4024,9 +4582,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{881ACF1F-DA10-4F3C-BBFE-3F6465156627}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>68</v>
       </c>
@@ -4037,7 +4595,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2018</v>
       </c>
@@ -4048,7 +4606,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2019</v>
       </c>
@@ -4059,7 +4617,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2020</v>
       </c>
@@ -4070,7 +4628,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2021</v>
       </c>
@@ -4081,7 +4639,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2022</v>
       </c>
@@ -4092,7 +4650,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2023</v>
       </c>
@@ -4103,7 +4661,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2024</v>
       </c>
@@ -4116,9 +4674,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80BA1C92-FA59-4C0B-BE43-3045F1F2387D}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>68</v>
       </c>
@@ -4129,7 +4687,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2018</v>
       </c>
@@ -4140,7 +4698,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2019</v>
       </c>
@@ -4151,7 +4709,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2020</v>
       </c>
@@ -4162,7 +4720,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2021</v>
       </c>
@@ -4173,7 +4731,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2022</v>
       </c>
@@ -4184,7 +4742,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2023</v>
       </c>
@@ -4195,7 +4753,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2024</v>
       </c>
@@ -4208,15 +4766,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BD10512-11B4-4E63-A14D-F810CE5069FA}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="23" customWidth="1"/>
-    <col min="3" max="3" width="17.85546875" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.28515625" customWidth="1"/>
+    <col min="3" max="3" width="17.88671875" customWidth="1"/>
+    <col min="4" max="4" width="11.44140625" customWidth="1"/>
+    <col min="5" max="5" width="10.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>68</v>
       </c>
@@ -4233,7 +4791,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2017</v>
       </c>
@@ -4250,7 +4808,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2018</v>
       </c>
@@ -4267,7 +4825,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2019</v>
       </c>
@@ -4284,7 +4842,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2020</v>
       </c>
@@ -4301,7 +4859,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2021</v>
       </c>
@@ -4318,7 +4876,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2022</v>
       </c>
@@ -4335,7 +4893,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2023</v>
       </c>
@@ -4352,7 +4910,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2024</v>
       </c>
@@ -4377,13 +4935,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26C20D99-1FC4-4882-8732-94F3CEFC30AD}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="17.5703125" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" customWidth="1"/>
+    <col min="4" max="4" width="17.5546875" customWidth="1"/>
+    <col min="5" max="5" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>68</v>
       </c>
@@ -4400,7 +4958,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2016</v>
       </c>
@@ -4417,7 +4975,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2017</v>
       </c>
@@ -4434,7 +4992,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2018</v>
       </c>
@@ -4451,7 +5009,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2019</v>
       </c>
@@ -4468,7 +5026,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2020</v>
       </c>
@@ -4485,7 +5043,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2021</v>
       </c>
@@ -4502,7 +5060,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2022</v>
       </c>
@@ -4519,7 +5077,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2023</v>
       </c>
@@ -4536,7 +5094,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2024</v>
       </c>
@@ -4561,13 +5119,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B540A97D-C280-43BD-9CE7-FD2678F34525}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="12.140625" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.109375" customWidth="1"/>
+    <col min="5" max="5" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>68</v>
       </c>
@@ -4584,7 +5142,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2016</v>
       </c>
@@ -4601,7 +5159,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2017</v>
       </c>
@@ -4618,7 +5176,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2018</v>
       </c>
@@ -4635,7 +5193,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2019</v>
       </c>
@@ -4652,7 +5210,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2020</v>
       </c>
@@ -4665,7 +5223,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2021</v>
       </c>
@@ -4682,7 +5240,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2022</v>
       </c>
@@ -4699,7 +5257,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2023</v>
       </c>
@@ -4716,7 +5274,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2024</v>
       </c>
@@ -4741,12 +5299,12 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A343A857-D05E-4917-9408-63BAE4D13234}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>68</v>
       </c>
@@ -4757,7 +5315,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2017</v>
       </c>
@@ -4768,7 +5326,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2018</v>
       </c>
@@ -4779,7 +5337,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2019</v>
       </c>
@@ -4790,7 +5348,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2020</v>
       </c>
@@ -4801,7 +5359,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2021</v>
       </c>
@@ -4812,7 +5370,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2022</v>
       </c>
@@ -4823,7 +5381,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2023</v>
       </c>
@@ -4834,7 +5392,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2024</v>
       </c>
@@ -4858,12 +5416,12 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{488D0083-044C-43F3-8315-2A23C120E975}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="17.5703125" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>68</v>
       </c>
@@ -4874,7 +5432,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2017</v>
       </c>
@@ -4885,7 +5443,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2018</v>
       </c>
@@ -4896,7 +5454,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2019</v>
       </c>
@@ -4907,7 +5465,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2020</v>
       </c>
@@ -4918,7 +5476,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2021</v>
       </c>
@@ -4929,7 +5487,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2022</v>
       </c>
@@ -4940,7 +5498,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2023</v>
       </c>
@@ -4951,7 +5509,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2024</v>
       </c>

</xml_diff>

<commit_message>
Added bridge maps, transit safety scorecards, and performance measure updates
</commit_message>
<xml_diff>
--- a/Performance_Measures_R.xlsx
+++ b/Performance_Measures_R.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://palmbeachtpa-my.sharepoint.com/personal/skan_palmbeachmpo_org/Documents/Documents/Performance_Measures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="541" documentId="8_{6E25A293-DAE1-403C-87C6-760DEF9E0950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3E5B97C-40A8-4DF4-AC5F-A859438403A2}"/>
+  <xr:revisionPtr revIDLastSave="548" documentId="8_{6E25A293-DAE1-403C-87C6-760DEF9E0950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9ED1DF6-AF79-4807-A69D-EEB27FF4B790}"/>
   <bookViews>
-    <workbookView xWindow="30315" yWindow="1515" windowWidth="21600" windowHeight="11295" activeTab="4" xr2:uid="{47865025-DE32-4D87-A21F-3C532F9D4B3D}"/>
+    <workbookView minimized="1" xWindow="30315" yWindow="1515" windowWidth="21600" windowHeight="11295" firstSheet="12" activeTab="20" xr2:uid="{47865025-DE32-4D87-A21F-3C532F9D4B3D}"/>
   </bookViews>
   <sheets>
     <sheet name="FATALITIES" sheetId="7" r:id="rId1"/>
     <sheet name="FATALITIES_5yr_avg" sheetId="35" r:id="rId2"/>
     <sheet name="SERIOUS INJURIES" sheetId="8" r:id="rId3"/>
     <sheet name="NM_Fat_Ser_Inj" sheetId="36" r:id="rId4"/>
-    <sheet name="Sheet1" sheetId="37" r:id="rId5"/>
+    <sheet name="Bridge_Main_Who" sheetId="37" r:id="rId5"/>
     <sheet name="PED FATINJ" sheetId="12" r:id="rId6"/>
     <sheet name="BIKE FATINJ" sheetId="13" r:id="rId7"/>
     <sheet name="BRIDGES" sheetId="14" r:id="rId8"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="151">
   <si>
     <t>Alachua</t>
   </si>
@@ -339,9 +339,6 @@
   </si>
   <si>
     <t>Bridges</t>
-  </si>
-  <si>
-    <t>Category</t>
   </si>
   <si>
     <t>Actual (2024)</t>
@@ -622,7 +619,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -668,9 +665,6 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1674,7 +1668,7 @@
         <v>68</v>
       </c>
       <c r="B1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C1" t="s">
         <v>78</v>
@@ -1786,7 +1780,7 @@
         <v>68</v>
       </c>
       <c r="B1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C1" t="s">
         <v>78</v>
@@ -1898,7 +1892,7 @@
         <v>68</v>
       </c>
       <c r="B1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C1" t="s">
         <v>78</v>
@@ -2010,7 +2004,7 @@
         <v>68</v>
       </c>
       <c r="B1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -2095,7 +2089,7 @@
         <v>68</v>
       </c>
       <c r="B1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C1" t="s">
         <v>78</v>
@@ -2182,7 +2176,7 @@
         <v>68</v>
       </c>
       <c r="B1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C1" t="s">
         <v>78</v>
@@ -2283,7 +2277,7 @@
         <v>68</v>
       </c>
       <c r="B1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -2357,7 +2351,7 @@
         <v>68</v>
       </c>
       <c r="B1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C1" t="s">
         <v>78</v>
@@ -2436,206 +2430,192 @@
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF8158D5-45CD-485F-9E37-C77E69A730F0}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B1" t="s">
-        <v>90</v>
+        <v>140</v>
       </c>
       <c r="C1" t="s">
         <v>141</v>
       </c>
-      <c r="D1" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="26" t="s">
-        <v>132</v>
-      </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>71</v>
       </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="26"/>
-      <c r="B3" t="s">
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>133</v>
+      </c>
+      <c r="B4">
+        <v>0.01</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B5">
+        <v>44</v>
+      </c>
+      <c r="C5">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>134</v>
       </c>
-      <c r="C3">
-        <v>0.01</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="26"/>
-      <c r="B4" t="s">
+      <c r="B6">
+        <v>0.1</v>
+      </c>
+      <c r="C6">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>135</v>
+      </c>
+      <c r="B7">
+        <v>49</v>
+      </c>
+      <c r="C7">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>136</v>
+      </c>
+      <c r="B8">
+        <v>0.6</v>
+      </c>
+      <c r="C8">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>137</v>
+      </c>
+      <c r="B9" s="22">
+        <v>7929</v>
+      </c>
+      <c r="C9" s="22">
+        <v>14000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>138</v>
+      </c>
+      <c r="B10" s="22"/>
+      <c r="C10" s="22"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>71</v>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>133</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>72</v>
       </c>
-      <c r="C4">
-        <v>44</v>
-      </c>
-      <c r="D4">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="26"/>
-      <c r="B5" t="s">
-        <v>135</v>
-      </c>
-      <c r="C5">
-        <v>0.1</v>
-      </c>
-      <c r="D5">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="26"/>
-      <c r="B6" t="s">
-        <v>136</v>
-      </c>
-      <c r="C6">
-        <v>49</v>
-      </c>
-      <c r="D6">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="26"/>
-      <c r="B7" t="s">
-        <v>137</v>
-      </c>
-      <c r="C7">
-        <v>0.6</v>
-      </c>
-      <c r="D7">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="26"/>
-      <c r="B8" t="s">
-        <v>138</v>
-      </c>
-      <c r="C8" s="22">
-        <v>7929</v>
-      </c>
-      <c r="D8" s="22">
-        <v>14000</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="26" t="s">
-        <v>139</v>
-      </c>
-      <c r="B9" t="s">
-        <v>71</v>
-      </c>
-      <c r="C9">
-        <v>0</v>
-      </c>
-      <c r="D9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="26"/>
-      <c r="B10" t="s">
+      <c r="B13">
+        <v>17</v>
+      </c>
+      <c r="C13">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>134</v>
       </c>
-      <c r="C10">
-        <v>0</v>
-      </c>
-      <c r="D10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="26"/>
-      <c r="B11" t="s">
-        <v>72</v>
-      </c>
-      <c r="C11">
-        <v>17</v>
-      </c>
-      <c r="D11">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="26"/>
-      <c r="B12" t="s">
-        <v>135</v>
-      </c>
-      <c r="C12">
+      <c r="B14">
         <v>0.2</v>
-      </c>
-      <c r="D12">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="26"/>
-      <c r="B13" t="s">
-        <v>136</v>
-      </c>
-      <c r="C13">
-        <v>17</v>
-      </c>
-      <c r="D13">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="26"/>
-      <c r="B14" t="s">
-        <v>137</v>
       </c>
       <c r="C14">
         <v>0.2</v>
       </c>
-      <c r="D14">
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>135</v>
+      </c>
+      <c r="B15">
+        <v>17</v>
+      </c>
+      <c r="C15">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>136</v>
+      </c>
+      <c r="B16">
         <v>0.2</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="26"/>
-      <c r="B15" t="s">
-        <v>138</v>
-      </c>
-      <c r="C15" s="22">
+      <c r="C16">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>137</v>
+      </c>
+      <c r="B17" s="22">
         <v>15101</v>
       </c>
-      <c r="D15" s="22">
+      <c r="C17" s="22">
         <v>7700</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:A8"/>
-    <mergeCell ref="A9:A15"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2650,7 +2630,7 @@
         <v>68</v>
       </c>
       <c r="B1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C1" t="s">
         <v>78</v>
@@ -2853,10 +2833,10 @@
         <v>89</v>
       </c>
       <c r="C1" t="s">
+        <v>92</v>
+      </c>
+      <c r="D1" t="s">
         <v>93</v>
-      </c>
-      <c r="D1" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -2866,41 +2846,41 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B3" t="s">
         <v>95</v>
-      </c>
-      <c r="B3" t="s">
-        <v>96</v>
       </c>
       <c r="C3" s="20">
         <v>0.83199999999999996</v>
       </c>
       <c r="D3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C4" s="20">
+        <v>0</v>
+      </c>
+      <c r="D4" t="s">
         <v>98</v>
-      </c>
-      <c r="B4" t="s">
-        <v>96</v>
-      </c>
-      <c r="C4" s="20">
-        <v>0</v>
-      </c>
-      <c r="D4" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="24" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C5" s="20"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B6" t="s">
         <v>83</v>
@@ -2909,49 +2889,49 @@
         <v>0.54700000000000004</v>
       </c>
       <c r="D6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C7" s="20">
         <v>0</v>
       </c>
       <c r="D7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C8" s="20">
         <v>0.56299999999999994</v>
       </c>
       <c r="D8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C9" s="20">
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="D9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -2977,15 +2957,15 @@
         <v>89</v>
       </c>
       <c r="C1" t="s">
+        <v>92</v>
+      </c>
+      <c r="D1" t="s">
         <v>93</v>
-      </c>
-      <c r="D1" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B2" t="s">
         <v>83</v>
@@ -2994,26 +2974,26 @@
         <v>0.623</v>
       </c>
       <c r="D2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C3" s="21">
         <v>0.86799999999999999</v>
       </c>
       <c r="D3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B4" t="s">
         <v>83</v>
@@ -3022,7 +3002,7 @@
         <v>2.09</v>
       </c>
       <c r="D4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -3046,65 +3026,65 @@
         <v>90</v>
       </c>
       <c r="B1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C1" t="s">
         <v>112</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>113</v>
-      </c>
-      <c r="D1" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B3" t="s">
+        <v>95</v>
+      </c>
+      <c r="C3" s="15">
+        <v>0</v>
+      </c>
+      <c r="D3" t="s">
         <v>116</v>
-      </c>
-      <c r="B3" t="s">
-        <v>96</v>
-      </c>
-      <c r="C3" s="15">
-        <v>0</v>
-      </c>
-      <c r="D3" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C4" s="15">
         <v>0</v>
       </c>
       <c r="D4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C5" s="15">
         <v>0</v>
       </c>
       <c r="D5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B6" t="s">
         <v>83</v>
@@ -3113,29 +3093,29 @@
         <v>0.434</v>
       </c>
       <c r="D6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C7" s="21">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="D7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C8" s="15">
         <v>0</v>
@@ -3146,14 +3126,14 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C9" s="15"/>
       <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B10" t="s">
         <v>83</v>
@@ -3162,49 +3142,49 @@
         <v>0.32</v>
       </c>
       <c r="D10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C11" s="15">
         <v>0.41</v>
       </c>
       <c r="D11" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>127</v>
+      </c>
+      <c r="B12" t="s">
+        <v>95</v>
+      </c>
+      <c r="C12" s="15">
+        <v>0</v>
+      </c>
+      <c r="D12" t="s">
         <v>128</v>
-      </c>
-      <c r="B12" t="s">
-        <v>96</v>
-      </c>
-      <c r="C12" s="15">
-        <v>0</v>
-      </c>
-      <c r="D12" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B13" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C13" s="21">
         <v>1.6000000000000001E-3</v>
       </c>
       <c r="D13" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -3228,18 +3208,18 @@
         <v>90</v>
       </c>
       <c r="B1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C1" t="s">
+        <v>92</v>
+      </c>
+      <c r="D1" t="s">
         <v>93</v>
-      </c>
-      <c r="D1" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -3247,7 +3227,7 @@
         <v>71</v>
       </c>
       <c r="B3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -3258,10 +3238,10 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C4">
         <v>0.01</v>
@@ -3275,7 +3255,7 @@
         <v>72</v>
       </c>
       <c r="B5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C5">
         <v>18</v>
@@ -3286,10 +3266,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C6">
         <v>0.2</v>
@@ -3300,10 +3280,10 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C7">
         <v>49</v>
@@ -3314,10 +3294,10 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C8">
         <v>0.7</v>
@@ -3328,10 +3308,10 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C9" s="22">
         <v>6609</v>
@@ -3342,7 +3322,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C10" s="22"/>
       <c r="D10" s="22"/>
@@ -3352,7 +3332,7 @@
         <v>71</v>
       </c>
       <c r="B11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -3363,10 +3343,10 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B12" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C12">
         <v>0</v>
@@ -3380,7 +3360,7 @@
         <v>72</v>
       </c>
       <c r="B13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C13">
         <v>20</v>
@@ -3391,10 +3371,10 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B14" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C14">
         <v>0.2</v>
@@ -3405,10 +3385,10 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B15" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C15">
         <v>14</v>
@@ -3419,10 +3399,10 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B16" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C16">
         <v>0.1</v>
@@ -3433,10 +3413,10 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B17" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C17" s="22">
         <v>10569</v>
@@ -5087,10 +5067,10 @@
         <v>68</v>
       </c>
       <c r="B1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C1" t="s">
         <v>144</v>
-      </c>
-      <c r="C1" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -5204,19 +5184,19 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
+        <v>145</v>
+      </c>
+      <c r="C1" t="s">
         <v>146</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>147</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>148</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>149</v>
-      </c>
-      <c r="F1" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -5241,7 +5221,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B3">
         <v>120516</v>

</xml_diff>

<commit_message>
fixed many small design details and uploading a prototype for review
</commit_message>
<xml_diff>
--- a/Performance_Measures_R.xlsx
+++ b/Performance_Measures_R.xlsx
@@ -8,39 +8,41 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://palmbeachtpa-my.sharepoint.com/personal/skan_palmbeachmpo_org/Documents/Documents/Performance_Measures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="548" documentId="8_{6E25A293-DAE1-403C-87C6-760DEF9E0950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9ED1DF6-AF79-4807-A69D-EEB27FF4B790}"/>
+  <xr:revisionPtr revIDLastSave="579" documentId="8_{6E25A293-DAE1-403C-87C6-760DEF9E0950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AA521C82-2B09-4D32-B438-B6DCDA49CF9A}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="30315" yWindow="1515" windowWidth="21600" windowHeight="11295" firstSheet="12" activeTab="20" xr2:uid="{47865025-DE32-4D87-A21F-3C532F9D4B3D}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="24" activeTab="28" xr2:uid="{47865025-DE32-4D87-A21F-3C532F9D4B3D}"/>
   </bookViews>
   <sheets>
     <sheet name="FATALITIES" sheetId="7" r:id="rId1"/>
     <sheet name="FATALITIES_5yr_avg" sheetId="35" r:id="rId2"/>
     <sheet name="SERIOUS INJURIES" sheetId="8" r:id="rId3"/>
-    <sheet name="NM_Fat_Ser_Inj" sheetId="36" r:id="rId4"/>
-    <sheet name="Bridge_Main_Who" sheetId="37" r:id="rId5"/>
-    <sheet name="PED FATINJ" sheetId="12" r:id="rId6"/>
-    <sheet name="BIKE FATINJ" sheetId="13" r:id="rId7"/>
-    <sheet name="BRIDGES" sheetId="14" r:id="rId8"/>
-    <sheet name="PAVEMENT INTERSTATE" sheetId="15" r:id="rId9"/>
-    <sheet name="PAVEMENT NON-INTERSTATE" sheetId="16" r:id="rId10"/>
-    <sheet name="TTTR Index" sheetId="17" r:id="rId11"/>
-    <sheet name="Int Reliability" sheetId="18" r:id="rId12"/>
-    <sheet name="Non-Int Reliability" sheetId="19" r:id="rId13"/>
-    <sheet name="UL_FRB" sheetId="26" r:id="rId14"/>
-    <sheet name="UL_CB" sheetId="27" r:id="rId15"/>
-    <sheet name="UL_SA" sheetId="28" r:id="rId16"/>
-    <sheet name="UL_ST" sheetId="29" r:id="rId17"/>
-    <sheet name="Trirail_Loco" sheetId="30" r:id="rId18"/>
-    <sheet name="Trirail_PER_R" sheetId="31" r:id="rId19"/>
-    <sheet name="Trirail_Sup_Main" sheetId="32" r:id="rId20"/>
-    <sheet name="PT_Safety_SC" sheetId="34" r:id="rId21"/>
-    <sheet name="Trirail_Facilties" sheetId="33" r:id="rId22"/>
-    <sheet name="Scorecard_Safety" sheetId="21" r:id="rId23"/>
-    <sheet name="Scorecard_Infrastructure" sheetId="22" r:id="rId24"/>
-    <sheet name="Scorecard_Sys_Per_Reli" sheetId="23" r:id="rId25"/>
-    <sheet name="Scorecard_Transit_As_Man" sheetId="24" r:id="rId26"/>
-    <sheet name="Scorecard_Transit_Safety" sheetId="25" r:id="rId27"/>
-    <sheet name="FATALITIES COMP" sheetId="3" state="hidden" r:id="rId28"/>
+    <sheet name="Sheet1" sheetId="38" r:id="rId4"/>
+    <sheet name="NM_Fat_Ser_Inj" sheetId="36" r:id="rId5"/>
+    <sheet name="Bridge_Main_Who" sheetId="37" r:id="rId6"/>
+    <sheet name="PED FATINJ" sheetId="12" r:id="rId7"/>
+    <sheet name="BIKE FATINJ" sheetId="13" r:id="rId8"/>
+    <sheet name="BRIDGES" sheetId="14" r:id="rId9"/>
+    <sheet name="PAVEMENT INTERSTATE" sheetId="15" r:id="rId10"/>
+    <sheet name="PAVEMENT NON-INTERSTATE" sheetId="16" r:id="rId11"/>
+    <sheet name="TTTR Index" sheetId="17" r:id="rId12"/>
+    <sheet name="Int Reliability" sheetId="18" r:id="rId13"/>
+    <sheet name="Non-Int Reliability" sheetId="19" r:id="rId14"/>
+    <sheet name="UL_FRB" sheetId="26" r:id="rId15"/>
+    <sheet name="UL_CB" sheetId="27" r:id="rId16"/>
+    <sheet name="UL_SA" sheetId="28" r:id="rId17"/>
+    <sheet name="UL_ST" sheetId="29" r:id="rId18"/>
+    <sheet name="Trirail_Loco" sheetId="30" r:id="rId19"/>
+    <sheet name="Trirail_PER_R" sheetId="31" r:id="rId20"/>
+    <sheet name="Trirail_Sup_Main" sheetId="32" r:id="rId21"/>
+    <sheet name="PT_Safety_SC" sheetId="34" r:id="rId22"/>
+    <sheet name="Trirail_Facilties" sheetId="33" r:id="rId23"/>
+    <sheet name="Scorecard_Safety" sheetId="21" r:id="rId24"/>
+    <sheet name="Scorecard_Infrastructure" sheetId="22" r:id="rId25"/>
+    <sheet name="Scorecard_Sys_Per_Reli" sheetId="23" r:id="rId26"/>
+    <sheet name="Scorecard_Transit_As_Man" sheetId="24" r:id="rId27"/>
+    <sheet name="Scorecard_Transit_Safety" sheetId="25" r:id="rId28"/>
+    <sheet name="Scorecard_All" sheetId="39" r:id="rId29"/>
+    <sheet name="FATALITIES COMP" sheetId="3" state="hidden" r:id="rId30"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -63,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="156">
   <si>
     <t>Alachua</t>
   </si>
@@ -516,6 +518,21 @@
   </si>
   <si>
     <t>Fair</t>
+  </si>
+  <si>
+    <t>SAFETY (5 -YR Avg.)</t>
+  </si>
+  <si>
+    <t>INFRASTRUCTURE</t>
+  </si>
+  <si>
+    <t>SYSTEM PERFORAMANCE RELIABILITY</t>
+  </si>
+  <si>
+    <t>TRANSIT ASSET MANAGEMENT</t>
+  </si>
+  <si>
+    <t>TRANSIT SAFETY: PALM TRAN</t>
   </si>
 </sst>
 </file>
@@ -1125,6 +1142,190 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26C20D99-1FC4-4882-8732-94F3CEFC30AD}">
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="17.5703125" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2016</v>
+      </c>
+      <c r="B2" s="14">
+        <v>0.62443452234924668</v>
+      </c>
+      <c r="C2" s="14">
+        <v>0</v>
+      </c>
+      <c r="D2" s="15">
+        <v>0.6</v>
+      </c>
+      <c r="E2" s="15">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2017</v>
+      </c>
+      <c r="B3" s="14">
+        <v>0.55162388800839957</v>
+      </c>
+      <c r="C3" s="14">
+        <v>0</v>
+      </c>
+      <c r="D3" s="15">
+        <v>0.6</v>
+      </c>
+      <c r="E3" s="15">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2018</v>
+      </c>
+      <c r="B4" s="14">
+        <v>0.23152561717146494</v>
+      </c>
+      <c r="C4" s="14">
+        <v>0</v>
+      </c>
+      <c r="D4" s="15">
+        <v>0.6</v>
+      </c>
+      <c r="E4" s="15">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2019</v>
+      </c>
+      <c r="B5" s="14">
+        <v>0.6120405364892294</v>
+      </c>
+      <c r="C5" s="14">
+        <v>0</v>
+      </c>
+      <c r="D5" s="15">
+        <v>0.6</v>
+      </c>
+      <c r="E5" s="15">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>2020</v>
+      </c>
+      <c r="B6" s="14">
+        <v>0.53156185428499947</v>
+      </c>
+      <c r="C6" s="14">
+        <v>2.3164663695412471E-3</v>
+      </c>
+      <c r="D6" s="15">
+        <v>0.6</v>
+      </c>
+      <c r="E6" s="15">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2021</v>
+      </c>
+      <c r="B7" s="14">
+        <v>0.59548474375249016</v>
+      </c>
+      <c r="C7" s="14">
+        <v>0</v>
+      </c>
+      <c r="D7" s="15">
+        <v>0.6</v>
+      </c>
+      <c r="E7" s="15">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>2022</v>
+      </c>
+      <c r="B8" s="14">
+        <v>0.64978966485364564</v>
+      </c>
+      <c r="C8" s="14">
+        <v>0</v>
+      </c>
+      <c r="D8" s="15">
+        <v>0.6</v>
+      </c>
+      <c r="E8" s="15">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>2023</v>
+      </c>
+      <c r="B9" s="14">
+        <v>0.67284019126365335</v>
+      </c>
+      <c r="C9" s="14">
+        <v>0</v>
+      </c>
+      <c r="D9" s="15">
+        <v>0.6</v>
+      </c>
+      <c r="E9" s="15">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>2024</v>
+      </c>
+      <c r="B10" s="14">
+        <v>0.54689337525889492</v>
+      </c>
+      <c r="C10" s="14">
+        <v>0</v>
+      </c>
+      <c r="D10" s="15">
+        <v>0.6</v>
+      </c>
+      <c r="E10" s="15">
+        <v>0.05</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B540A97D-C280-43BD-9CE7-FD2678F34525}">
   <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1304,7 +1505,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A343A857-D05E-4917-9408-63BAE4D13234}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1421,7 +1622,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{488D0083-044C-43F3-8315-2A23C120E975}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1538,7 +1739,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CB9C645-8F86-45BC-BA51-DC3AF3602CC7}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1655,7 +1856,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70545EE8-3393-48FF-8B94-A68F78870296}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1767,7 +1968,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8768E2E-41F2-4128-AF4B-DB787856BFE5}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1879,7 +2080,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47C9403F-1360-4C9E-9A0D-37F31FFD517C}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1991,7 +2192,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F62C98EA-F049-4A45-95E1-AA425574422A}">
   <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2076,7 +2277,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDBE33F8-F6FD-46D3-B669-CD9D8BFF9D18}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2159,104 +2360,6 @@
       </c>
       <c r="C7" s="15">
         <v>0.28599999999999998</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2012453B-2FD9-4676-A93F-5D42E7C311A7}">
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B1" t="s">
-        <v>139</v>
-      </c>
-      <c r="C1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>2018</v>
-      </c>
-      <c r="B2" s="15">
-        <v>0.08</v>
-      </c>
-      <c r="C2" s="15">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2019</v>
-      </c>
-      <c r="B3" s="23">
-        <v>3.3000000000000002E-2</v>
-      </c>
-      <c r="C3" s="15">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>2020</v>
-      </c>
-      <c r="B4" s="23">
-        <v>0</v>
-      </c>
-      <c r="C4" s="15">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>2021</v>
-      </c>
-      <c r="B5" s="23">
-        <v>2.1000000000000001E-2</v>
-      </c>
-      <c r="C5" s="15">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>2022</v>
-      </c>
-      <c r="B6" s="23">
-        <v>1.5E-3</v>
-      </c>
-      <c r="C6" s="15">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>2023</v>
-      </c>
-      <c r="B7" s="23">
-        <v>1.6000000000000001E-3</v>
-      </c>
-      <c r="C7" s="15">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>2024</v>
-      </c>
-      <c r="B8" s="23">
-        <v>1.6000000000000001E-3</v>
-      </c>
-      <c r="C8" s="15">
-        <v>0.03</v>
       </c>
     </row>
   </sheetData>
@@ -2342,6 +2445,104 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2012453B-2FD9-4676-A93F-5D42E7C311A7}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2018</v>
+      </c>
+      <c r="B2" s="15">
+        <v>0.08</v>
+      </c>
+      <c r="C2" s="15">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2019</v>
+      </c>
+      <c r="B3" s="23">
+        <v>3.3000000000000002E-2</v>
+      </c>
+      <c r="C3" s="15">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2020</v>
+      </c>
+      <c r="B4" s="23">
+        <v>0</v>
+      </c>
+      <c r="C4" s="15">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2021</v>
+      </c>
+      <c r="B5" s="23">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="C5" s="15">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>2022</v>
+      </c>
+      <c r="B6" s="23">
+        <v>1.5E-3</v>
+      </c>
+      <c r="C6" s="15">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2023</v>
+      </c>
+      <c r="B7" s="23">
+        <v>1.6000000000000001E-3</v>
+      </c>
+      <c r="C7" s="15">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>2024</v>
+      </c>
+      <c r="B8" s="23">
+        <v>1.6000000000000001E-3</v>
+      </c>
+      <c r="C8" s="15">
+        <v>0.03</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBB831B4-CACE-4DDE-9F5D-2A702D15F4A9}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2428,7 +2629,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF8158D5-45CD-485F-9E37-C77E69A730F0}">
   <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2620,7 +2821,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8A2B925-F3EE-472B-B53C-CA468800D579}">
   <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2718,7 +2919,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B420F60-609B-4AA9-97E6-C695A4A591CA}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2816,7 +3017,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B84F7EA7-DBFB-4CBA-A1A1-E112D361DAFF}">
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2939,7 +3140,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8FF0919-3905-4425-81BF-3149EAA458D8}">
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3010,7 +3211,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1963ABED-C249-4004-B31E-6E99DC2E6917}">
   <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3192,7 +3393,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C3051EB-9F2E-4379-8AFD-5E4458A288D3}">
   <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3430,7 +3631,727 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A80654F7-7F84-4744-9CA4-C221A28D6B22}">
+  <dimension ref="A1:D50"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="54.85546875" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1" t="s">
+        <v>92</v>
+      </c>
+      <c r="D1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="24" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C3">
+        <v>207.4</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4">
+        <v>1.45</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C5">
+        <v>812.2</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>85</v>
+      </c>
+      <c r="B6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6">
+        <v>5.73</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C7">
+        <v>203.8</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="24" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="24" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>94</v>
+      </c>
+      <c r="B10" t="s">
+        <v>95</v>
+      </c>
+      <c r="C10" s="20">
+        <v>0.83199999999999996</v>
+      </c>
+      <c r="D10" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>97</v>
+      </c>
+      <c r="B11" t="s">
+        <v>95</v>
+      </c>
+      <c r="C11" s="20">
+        <v>0</v>
+      </c>
+      <c r="D11" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="24" t="s">
+        <v>99</v>
+      </c>
+      <c r="C12" s="20"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>100</v>
+      </c>
+      <c r="B13" t="s">
+        <v>83</v>
+      </c>
+      <c r="C13" s="20">
+        <v>0.54700000000000004</v>
+      </c>
+      <c r="D13" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>102</v>
+      </c>
+      <c r="B14" t="s">
+        <v>95</v>
+      </c>
+      <c r="C14" s="20">
+        <v>0</v>
+      </c>
+      <c r="D14" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>103</v>
+      </c>
+      <c r="B15" t="s">
+        <v>95</v>
+      </c>
+      <c r="C15" s="20">
+        <v>0.56299999999999994</v>
+      </c>
+      <c r="D15" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>105</v>
+      </c>
+      <c r="B16" t="s">
+        <v>95</v>
+      </c>
+      <c r="C16" s="20">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="D16" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="24" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>106</v>
+      </c>
+      <c r="B18" t="s">
+        <v>83</v>
+      </c>
+      <c r="C18" s="21">
+        <v>0.623</v>
+      </c>
+      <c r="D18" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>108</v>
+      </c>
+      <c r="B19" t="s">
+        <v>95</v>
+      </c>
+      <c r="C19" s="21">
+        <v>0.86799999999999999</v>
+      </c>
+      <c r="D19" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>109</v>
+      </c>
+      <c r="B20" t="s">
+        <v>83</v>
+      </c>
+      <c r="C20">
+        <v>2.09</v>
+      </c>
+      <c r="D20" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="24" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="24" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>115</v>
+      </c>
+      <c r="B23" t="s">
+        <v>95</v>
+      </c>
+      <c r="C23" s="15">
+        <v>0</v>
+      </c>
+      <c r="D23" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>117</v>
+      </c>
+      <c r="B24" t="s">
+        <v>95</v>
+      </c>
+      <c r="C24" s="15">
+        <v>0</v>
+      </c>
+      <c r="D24" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>118</v>
+      </c>
+      <c r="B25" t="s">
+        <v>95</v>
+      </c>
+      <c r="C25" s="15">
+        <v>0</v>
+      </c>
+      <c r="D25" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>119</v>
+      </c>
+      <c r="B26" t="s">
+        <v>83</v>
+      </c>
+      <c r="C26" s="21">
+        <v>0.434</v>
+      </c>
+      <c r="D26" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>120</v>
+      </c>
+      <c r="B27" t="s">
+        <v>95</v>
+      </c>
+      <c r="C27" s="21">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="D27" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>121</v>
+      </c>
+      <c r="B28" t="s">
+        <v>95</v>
+      </c>
+      <c r="C28" s="15">
+        <v>0</v>
+      </c>
+      <c r="D28" s="15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="24" t="s">
+        <v>122</v>
+      </c>
+      <c r="C29" s="15"/>
+      <c r="D29" s="15"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>123</v>
+      </c>
+      <c r="B30" t="s">
+        <v>83</v>
+      </c>
+      <c r="C30" s="15">
+        <v>0.32</v>
+      </c>
+      <c r="D30" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>125</v>
+      </c>
+      <c r="B31" t="s">
+        <v>95</v>
+      </c>
+      <c r="C31" s="15">
+        <v>0.41</v>
+      </c>
+      <c r="D31" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>127</v>
+      </c>
+      <c r="B32" t="s">
+        <v>95</v>
+      </c>
+      <c r="C32" s="15">
+        <v>0</v>
+      </c>
+      <c r="D32" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>129</v>
+      </c>
+      <c r="B33" t="s">
+        <v>95</v>
+      </c>
+      <c r="C33" s="21">
+        <v>1.6000000000000001E-3</v>
+      </c>
+      <c r="D33" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="24" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>71</v>
+      </c>
+      <c r="B36" t="s">
+        <v>132</v>
+      </c>
+      <c r="C36">
+        <v>1</v>
+      </c>
+      <c r="D36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>133</v>
+      </c>
+      <c r="B37" t="s">
+        <v>132</v>
+      </c>
+      <c r="C37">
+        <v>0.01</v>
+      </c>
+      <c r="D37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>72</v>
+      </c>
+      <c r="B38" t="s">
+        <v>132</v>
+      </c>
+      <c r="C38">
+        <v>18</v>
+      </c>
+      <c r="D38">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>134</v>
+      </c>
+      <c r="B39" t="s">
+        <v>132</v>
+      </c>
+      <c r="C39">
+        <v>0.2</v>
+      </c>
+      <c r="D39">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>135</v>
+      </c>
+      <c r="B40" t="s">
+        <v>132</v>
+      </c>
+      <c r="C40">
+        <v>49</v>
+      </c>
+      <c r="D40">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>136</v>
+      </c>
+      <c r="B41" t="s">
+        <v>132</v>
+      </c>
+      <c r="C41">
+        <v>0.7</v>
+      </c>
+      <c r="D41">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>137</v>
+      </c>
+      <c r="B42" t="s">
+        <v>132</v>
+      </c>
+      <c r="C42" s="22">
+        <v>6609</v>
+      </c>
+      <c r="D42" s="22">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="24" t="s">
+        <v>138</v>
+      </c>
+      <c r="C43" s="22"/>
+      <c r="D43" s="22"/>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>71</v>
+      </c>
+      <c r="B44" t="s">
+        <v>132</v>
+      </c>
+      <c r="C44">
+        <v>0</v>
+      </c>
+      <c r="D44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>133</v>
+      </c>
+      <c r="B45" t="s">
+        <v>132</v>
+      </c>
+      <c r="C45">
+        <v>0</v>
+      </c>
+      <c r="D45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>72</v>
+      </c>
+      <c r="B46" t="s">
+        <v>132</v>
+      </c>
+      <c r="C46">
+        <v>20</v>
+      </c>
+      <c r="D46">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>134</v>
+      </c>
+      <c r="B47" t="s">
+        <v>132</v>
+      </c>
+      <c r="C47">
+        <v>0.2</v>
+      </c>
+      <c r="D47">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>135</v>
+      </c>
+      <c r="B48" t="s">
+        <v>132</v>
+      </c>
+      <c r="C48">
+        <v>14</v>
+      </c>
+      <c r="D48">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>136</v>
+      </c>
+      <c r="B49" t="s">
+        <v>132</v>
+      </c>
+      <c r="C49">
+        <v>0.1</v>
+      </c>
+      <c r="D49">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>137</v>
+      </c>
+      <c r="B50" t="s">
+        <v>132</v>
+      </c>
+      <c r="C50" s="22">
+        <v>10569</v>
+      </c>
+      <c r="D50" s="22">
+        <v>7700</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{504C1906-E774-4362-B18C-74A3CE45CFF8}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="14.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2018</v>
+      </c>
+      <c r="B2" s="9">
+        <v>1194</v>
+      </c>
+      <c r="C2" s="8">
+        <v>8.42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2019</v>
+      </c>
+      <c r="B3" s="9">
+        <v>1020</v>
+      </c>
+      <c r="C3" s="8">
+        <v>7.08</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2020</v>
+      </c>
+      <c r="B4" s="10">
+        <v>916</v>
+      </c>
+      <c r="C4" s="8">
+        <v>6.91</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2021</v>
+      </c>
+      <c r="B5" s="10">
+        <v>890</v>
+      </c>
+      <c r="C5" s="8">
+        <v>6.45</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>2022</v>
+      </c>
+      <c r="B6" s="10">
+        <v>818</v>
+      </c>
+      <c r="C6" s="8">
+        <v>5.73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2023</v>
+      </c>
+      <c r="B7" s="10">
+        <v>766</v>
+      </c>
+      <c r="C7" s="8">
+        <v>5.16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>2024</v>
+      </c>
+      <c r="B8" s="7">
+        <v>683</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DE6782D-92DC-4DC3-BB49-53C081EF8C06}">
   <dimension ref="A1:BP8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4956,105 +5877,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{504C1906-E774-4362-B18C-74A3CE45CFF8}">
-  <dimension ref="A1:C8"/>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A79765B-4EBA-4E5D-B48C-B122FB21D217}">
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="14.5703125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B1" t="s">
-        <v>69</v>
-      </c>
-      <c r="C1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>2018</v>
-      </c>
-      <c r="B2" s="9">
-        <v>1194</v>
-      </c>
-      <c r="C2" s="8">
-        <v>8.42</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2019</v>
-      </c>
-      <c r="B3" s="9">
-        <v>1020</v>
-      </c>
-      <c r="C3" s="8">
-        <v>7.08</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>2020</v>
-      </c>
-      <c r="B4" s="10">
-        <v>916</v>
-      </c>
-      <c r="C4" s="8">
-        <v>6.91</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>2021</v>
-      </c>
-      <c r="B5" s="10">
-        <v>890</v>
-      </c>
-      <c r="C5" s="8">
-        <v>6.45</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>2022</v>
-      </c>
-      <c r="B6" s="10">
-        <v>818</v>
-      </c>
-      <c r="C6" s="8">
-        <v>5.73</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>2023</v>
-      </c>
-      <c r="B7" s="10">
-        <v>766</v>
-      </c>
-      <c r="C7" s="8">
-        <v>5.16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>2024</v>
-      </c>
-      <c r="B8" s="7">
-        <v>683</v>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E6E1516-3CB9-4A84-B657-9470D488082C}">
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5177,7 +6009,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72932D94-618B-4319-8748-A0A0A4D4F4C7}">
   <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5264,7 +6096,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{881ACF1F-DA10-4F3C-BBFE-3F6465156627}">
   <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5356,7 +6188,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80BA1C92-FA59-4C0B-BE43-3045F1F2387D}">
   <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5448,7 +6280,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BD10512-11B4-4E63-A14D-F810CE5069FA}">
   <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5615,188 +6447,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26C20D99-1FC4-4882-8732-94F3CEFC30AD}">
-  <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="4" max="4" width="17.5703125" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D1" t="s">
-        <v>82</v>
-      </c>
-      <c r="E1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>2016</v>
-      </c>
-      <c r="B2" s="14">
-        <v>0.62443452234924668</v>
-      </c>
-      <c r="C2" s="14">
-        <v>0</v>
-      </c>
-      <c r="D2" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="E2" s="15">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2017</v>
-      </c>
-      <c r="B3" s="14">
-        <v>0.55162388800839957</v>
-      </c>
-      <c r="C3" s="14">
-        <v>0</v>
-      </c>
-      <c r="D3" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="E3" s="15">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>2018</v>
-      </c>
-      <c r="B4" s="14">
-        <v>0.23152561717146494</v>
-      </c>
-      <c r="C4" s="14">
-        <v>0</v>
-      </c>
-      <c r="D4" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="E4" s="15">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>2019</v>
-      </c>
-      <c r="B5" s="14">
-        <v>0.6120405364892294</v>
-      </c>
-      <c r="C5" s="14">
-        <v>0</v>
-      </c>
-      <c r="D5" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="E5" s="15">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>2020</v>
-      </c>
-      <c r="B6" s="14">
-        <v>0.53156185428499947</v>
-      </c>
-      <c r="C6" s="14">
-        <v>2.3164663695412471E-3</v>
-      </c>
-      <c r="D6" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="E6" s="15">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>2021</v>
-      </c>
-      <c r="B7" s="14">
-        <v>0.59548474375249016</v>
-      </c>
-      <c r="C7" s="14">
-        <v>0</v>
-      </c>
-      <c r="D7" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="E7" s="15">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>2022</v>
-      </c>
-      <c r="B8" s="14">
-        <v>0.64978966485364564</v>
-      </c>
-      <c r="C8" s="14">
-        <v>0</v>
-      </c>
-      <c r="D8" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="E8" s="15">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>2023</v>
-      </c>
-      <c r="B9" s="14">
-        <v>0.67284019126365335</v>
-      </c>
-      <c r="C9" s="14">
-        <v>0</v>
-      </c>
-      <c r="D9" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="E9" s="15">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>2024</v>
-      </c>
-      <c r="B10" s="14">
-        <v>0.54689337525889492</v>
-      </c>
-      <c r="C10" s="14">
-        <v>0</v>
-      </c>
-      <c r="D10" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="E10" s="15">
-        <v>0.05</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>